<commit_message>
Pesan commit yang menjelaskan perubahan
</commit_message>
<xml_diff>
--- a/data/outputs/1. IVC DOE R2 (Final).xlsx
+++ b/data/outputs/1. IVC DOE R2 (Final).xlsx
@@ -508,43 +508,51 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>I am ready to proceed. Please provide the raw input text containing the 'Risk Description' you would like me to summarize.</t>
+          <t>Risk related to RBS Level 1 categorization with potential technical or design implications.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Rbs Level 1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Lead engineer</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Mitigating Action:</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+          <t>The Lead engineer should review and validate the RBS Level 1 categorization to ensure proper risk alignment and mitigation planning.</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -554,12 +562,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R4.6</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Data sharing from BBSRI at risk.</t>
+          <t>Data sharing from BBSRI for smolt probability of encounter model is at risk, potentially hindering environmental monitoring plan development.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -569,7 +577,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Regulations</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -578,24 +586,32 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Facilitate conversations with Umaine on data sharing</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+          <t>Facilitate conversations between LGL, BBSRI, and Umaine regarding data sharing agreements.</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -605,22 +621,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ice data collection may be unsuccessful.</t>
+          <t>Ice data collection may be unsuccessful, requiring equipment retrieval and redeployment.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Pre-construction</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Stakeholder</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -629,24 +645,32 @@
         </is>
       </c>
       <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Implement real-time data collection and have UAF lead the technical side with continued management oversight.</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
         <v>2</v>
       </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>real time data collection implemented</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -656,22 +680,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FERC license not granted in time, risking schedule slip and budget creep.</t>
+          <t>FERC license may not be granted in time for open water testing, causing schedule slip and budget creep.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Regulations</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -680,7 +704,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
         <v>4</v>
@@ -692,12 +716,20 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Initiate communication with Regulatory agencies and FERC to scope FERC License. Resource appropriately for completion by 12/17, respond to Additional Information Requests promptly after submission</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+          <t>Initiate communication with Regulatory agencies and FERC to scope the FERC License, resource appropriately for completion by 12/17, and respond to Additional Information Requests promptly after submission.</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -707,12 +739,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wet Gap Generator design not yet complete.</t>
+          <t>Wet Gap Generator design not yet complete, risking manufactured product being out of specification and causing increased cost/schedule slip.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -734,7 +766,7 @@
         <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -743,12 +775,20 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Design reviews and component validation testing before design finalized</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+          <t>Work closely with Generator vendor to develop clear specification and ensure generator design meets this specification through design reviews and component validation testing.</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -758,12 +798,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tight generator procurement timing risks project schedule.</t>
+          <t>Timing of generator procurement from IKM could be tight for schedule, potentially leading to manufacturing or integration issues that need resolution in a limited time frame.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -773,7 +813,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -785,7 +825,7 @@
         <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -794,12 +834,20 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Ensure Generator delivery by 2/2018 to allow adequate time for testing using project development plan with regular status reports</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+          <t>Ensure Generator delivery by 2/2018 to allow adequate time for testing using project development plan with regular status reports and continue communication with IKM and ORPC Ireland to ensure timely procurement.</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -809,22 +857,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Unexpected component shortage may delay buoyancy system validation tests.</t>
+          <t>Unexpected component shortages in buoyancy system procurement could delay validation tests.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -833,10 +881,10 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -845,12 +893,20 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Compile BOM and ascertain component lead times from vendors in advance of PO issue</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+          <t>Compile BOM and ascertain component lead times from vendors in advance of PO issue.</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -860,17 +916,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fabricated components have significant lead times.</t>
+          <t>Fabricated components have significant lead times, causing unexpected fabrication delays that increase cost and effort.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -884,7 +940,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
         <v>6</v>
@@ -896,12 +952,20 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Frequent vendor communication, issue PO with room for schedule creep, rapid change order resolution, contractual penalties for schedule slip</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+          <t>Implement frequent vendor communications, issue POs with schedule flexibility, rapid change order resolution, and include contractual penalties for late delivery.</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -911,22 +975,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fabricated components have significant lead times, risking project schedule.</t>
+          <t>Fabricated components have significant lead times, risking unexpected fabrication delays, increased costs, and effort.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -935,10 +999,10 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -947,12 +1011,20 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Frequent vendor communication, issue PO with room for schedule creep, rapid change order resolution, contractual penalties for schedule slip</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+          <t>Implement frequent vendor communication, issue POs with schedule flexibility, and include contractual penalties for late delivery.</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -962,22 +1034,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Single-source vendor dependency risks design completion and fabrication delays.</t>
+          <t>Single source vendor for critical components creates dependency risks during design completion and fabrication phases.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -989,21 +1061,29 @@
         <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Frequent vendor communication, issue PO with room for schedule creep, rapid change order resolution, contractual penalties for schedule slip</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+          <t>Implement frequent vendor communications, issue PO with schedule flexibility, establish rapid change order resolution, and include contractual penalties for delivery delays.</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1013,22 +1093,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Unexpected component shortages or personnel shortages for SCADA development may delay integration and system validation.</t>
+          <t>Unexpected component or personnel shortages delay SCADA system procurement, integration, and validation.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1040,7 +1120,7 @@
         <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1049,12 +1129,20 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Compile BOM and ascertain component lead times from vendors in advance of PO issue</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+          <t>Compile a Bill of Materials and verify component lead times with vendors before issuing purchase orders.</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1064,17 +1152,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fabrication delays and out-of-spec delivered product from suppliers.</t>
+          <t>Fabrication delays and out-of-spec delivered product from suppliers/vendors during power and data cable procurement.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1091,7 +1179,7 @@
         <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1100,12 +1188,20 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Compile BOM and ascertain component lead times from vendors in advance of PO issue</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+          <t>Compile BOM and ascertain component lead times from vendors in advance of PO issue, and use COTS components where possible.</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1115,22 +1211,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Unexpected component shortage may delay mooring system validation tests.</t>
+          <t>Unexpected component shortages in mooring system procurement could delay validation tests.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1151,12 +1247,20 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Compile BOM and ascertain component lead times from vendors in advance of PO issue</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+          <t>Compile bill of materials and verify component lead times with vendors before purchase order issuance.</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1166,22 +1270,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Custom components require fabrication lead time.</t>
+          <t>Custom components require fabrication lead time, potentially causing unexpected delays and increased costs.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1193,7 +1297,7 @@
         <v>3</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1202,12 +1306,20 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Frequent vendor communication, issue PO with room for schedule creep, rapid change order resolution, contractual penalties for schedule slip or incorrect product delivery</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+          <t>Implement frequent vendor communications, issue POs with schedule flexibility, and include contractual penalties for late delivery.</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1217,22 +1329,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Custom components require fabrication lead time, risking project schedule and budget.</t>
+          <t>Custom components require fabrication lead time, potentially causing unexpected delays and increased costs.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1244,7 +1356,7 @@
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1253,12 +1365,20 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Frequent vendor communication, issue PO with room for schedule creep, rapid change order resolution, contractual penalties for schedule slip or incorrect product delivery</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+          <t>Implement frequent vendor communication, issue PO with schedule buffer, and include contractual penalties for late delivery.</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1268,17 +1388,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Buoyancy system fails validation tests, risking project schedule and requiring redesign.</t>
+          <t>Buoyancy System fails some or all of validation tests, potentially leading to unexpected component failure after validation but prior to deployment.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1295,7 +1415,7 @@
         <v>3</v>
       </c>
       <c r="H17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1304,12 +1424,20 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Utilizing incremental improvements to a proven concept, add redundancy to design. Perform land based tests in May 2017 and move on to on water validation tests prior to shipment to Igiugig.</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+          <t>Utilize incremental improvements to a proven concept, add redundancy to design, perform land-based tests in May 2017, and conduct on-water validation tests prior to shipment to Igiugig.</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1319,17 +1447,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Structural assembly may fail validation tests, risking project integrity and costs.</t>
+          <t>Structural assembly fails some or all validation tests during testing phases.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1355,12 +1483,20 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>FEA analysis following DNV standards, detailed CAD validation, and incorporate structural redundancy.</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+          <t>Perform FEA analysis following DNV standards, incorporate structural redundancy, and conduct thorough validation tests before assembly.</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>4</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1370,17 +1506,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Turbine assembly may fail validation tests, leading to unexpected failure or reduced performance.</t>
+          <t>Turbine assembly fails some or all validation tests during assembly and commissioning.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1394,24 +1530,32 @@
         </is>
       </c>
       <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Utilize CFD and FEA analysis following DNV standards and incorporate third-party design review.</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
         <v>2</v>
       </c>
-      <c r="H19" t="n">
-        <v>6</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Utilize CFD as design tool for performance validation, FEA analysis of turbines include load factors following DNV standards and considers extreme loading conditions, secondary design input from composite manufacturer</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1421,17 +1565,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Generator fails validation tests, risking project schedule and costs.</t>
+          <t>Generator fails some or all validation tests, leading to unexpected failure, increased costs, and schedule slippage.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1445,10 +1589,10 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1457,12 +1601,20 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Factory Acceptance testing and laboratory testing of Generator integrated with Power electronics to ensure compatibility before assembly and commissioning</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+          <t>Conduct Factory Acceptance Testing and laboratory testing of the Generator integrated with Power electronics to ensure compatibility before assembly and commissioning.</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1472,17 +1624,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Power Electronics fails validation, risking project schedule and costs.</t>
+          <t>Power Electronics fails validation, potentially leading to unexpected failure or grid integration issues.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1499,21 +1651,29 @@
         <v>3</v>
       </c>
       <c r="H21" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Factory acceptance tests and sequenced laboratory testing to ensure Power Electronics meets requirements before shipment</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
+          <t>Conduct factory acceptance tests and sequenced laboratory testing to ensure Power Electronics meets requirements before shipment.</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
+        <v>3</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1523,17 +1683,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SCADA system fails validation.</t>
+          <t>SCADA system fails validation, potentially leading to unexpected failures or communication issues during operation.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1550,7 +1710,7 @@
         <v>3</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1559,12 +1719,20 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Factory acceptance tests and sequenced laboratory testing to ensure SCADA meets requirements before shipment</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
+          <t>Conduct factory acceptance tests and sequenced laboratory testing to ensure SCADA meets requirements before shipment.</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1574,17 +1742,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Unexpected power and data cable failure.</t>
+          <t>Power and data cables failure during multiple project phases.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1601,21 +1769,29 @@
         <v>4</v>
       </c>
       <c r="H23" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Utilize proven cable technology, secondary cable armor in high risk areas, redundant conductors for data and fiber optic, reduce inspections and associated wear and tear</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+          <t>Utilize proven cable technology with secondary armor and redundant conductors, and test full length cable with SCADA system.</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1625,17 +1801,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mooring system failure due to inadequate design or validation.</t>
+          <t>Mooring system failure due to inadequate design or component specification.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1661,12 +1837,20 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Design to DNV standards, utilize geophysical knowledge and industry expertise to specify mooring system components, consider most favorable failure modes.</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+          <t>Design to DNV standards, utilize geophysical knowledge, and seek industry expertise to specify mooring system components considering favorable failure modes.</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" t="n">
+        <v>4</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1676,17 +1860,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Driveline failure risk requiring validation testing and design for increased tolerances.</t>
+          <t>Driveline failure due to inadequate validation testing and design tolerances.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1700,7 +1884,7 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H25" t="n">
         <v>4</v>
@@ -1712,12 +1896,20 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Thorough validation testing, design for increased tolerances and loads, choose long-life low-maintenance components, increase modularity.</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
+          <t>Conduct thorough validation testing before assembly and commissioning, incorporate design modifications for increased operational tolerances and modularity.</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" t="n">
+        <v>3</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1727,17 +1919,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mechanical brake failure risk requiring validation and redundant electrical brake.</t>
+          <t>Mechanical brake failure could occur during multiple project phases, requiring reliance on redundant electrical systems.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1763,12 +1955,20 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Thorough validation testing including redundant electrical brake</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+          <t>Complete thorough validation testing including redundant electrical brake system implementation.</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1783,17 +1983,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Delays in receiving FERC pilot licenses or permits compromise project deployment.</t>
+          <t>Receipt of FERC pilot license or permits are delayed and compromise deployment due to uncertainty with regulatory agency approvals.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Pre-construction</t>
+          <t>Multiple (Or All) Life Phases</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Regulations</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1802,10 +2002,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1814,12 +2014,20 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Continue regular dialogue with regulatory agencies after final pilot license and other permit applications, respond to AIRs in timely manner</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
+          <t>Continue regular dialogue with regulatory agencies after final pilot license and other permit applications, and respond to AIRs in a timely manner.</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>3</v>
+      </c>
+      <c r="L27" t="n">
+        <v>3</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1829,17 +2037,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Component shipment to Igiugig is delayed due to schedule slip, transportation contractor issues, weather, or other factors.</t>
+          <t>Component shipment to Igiugig is delayed due to schedule slip, transportation contractor issues, weather or other factors.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1856,21 +2064,29 @@
         <v>4</v>
       </c>
       <c r="H28" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Track project schedule, align component validation and delivery to port of shipment with shipper schedules, ship components early if possible arrival on first barge of season (June 2018) or second (July 2018) at latest</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
+          <t>Track project schedule, align component validation and delivery to port of shipment with shipper schedules, and ship components early if possible for arrival on first or second barge of season.</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1880,12 +2096,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Device assembly may be difficult or require modification in Igiugig.</t>
+          <t>Device assembly is difficult or requires modification in Igiugig due to component interfaces, damage during shipment, or other issues during June-August 2018.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,21 +2123,29 @@
         <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Preassemble components prior to shipment; include assembly in validation.</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
+          <t>Preassemble as many components as possible prior to shipment to Igiugig to reduce on-site assembly steps and costs.</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1931,12 +2155,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Power system deployment and commissioning may encounter unexpected difficulties.</t>
+          <t>Power System deployment/commissioning encounters unexpected difficulties during assembly and commissioning.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1955,10 +2179,10 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1967,12 +2191,20 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>prior device testing and component testing in Nikiksi and elsewhere will reduce unexpected issues with deployment or comissioning. Thewe validation steps completed by May 2018</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+          <t>Test all components in configuration for Igiugig deployment when practical and within budget.</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
+        <v>4</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1987,12 +2219,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ice accumulation or interaction with device causes power disruption, reduction, or equipment damage.</t>
+          <t>Ice accumulation on or interaction with the device causes power disruption, reduction, or equipment damage.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Extreme Events</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2009,7 +2241,7 @@
         <v>3</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2018,12 +2250,20 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Collection of in river ice data for 2 years prior to deployment feeds engineering and IO&amp;M planning, June 2017- June 2018. On device ice monitoring allows for operational state modification if adverse conditions or interactions occur.</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+          <t>Perform thorough analysis of ice data from in-river data collection and conduct a thorough FMEA of risks this type of ice formation or movement will have on the device.</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
+        <v>4</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2038,43 +2278,51 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Adverse salmon smolt interactions during device operation.</t>
+          <t>Salmon smolt data collection may show adverse interactions or be inadequate for regulatory approval, potentially halting device operation during outmigration.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Normal Power Production</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>Environmental</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Environmental</t>
-        </is>
-      </c>
       <c r="G32" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H32" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Develop rigorous fish monitoring plan in budget period 2, consult with agencies regularly, operate device only under continuous monitoring during smolt outmigration</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+          <t>Develop a rigorous fish monitoring plan in consultation with state and federal agencies to ensure adequate data collection for operational decisions during smolt outmigration.</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>3</v>
+      </c>
+      <c r="L32" t="n">
+        <v>4</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2084,12 +2332,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Device removal complicated by technological or environmental factors.</t>
+          <t>Device removal is complicated by technological or environmental factors during decommissioning.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2120,12 +2368,20 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Buoyancy system includes redundant and isolated retrieval mechanisms, pre-testing in Nikiski to reduce risk of retrieval issues arising.</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
+          <t>Implement redundant and isolated retrieval mechanisms with pre-testing in Nikiski to reduce the likelihood of retrieval issues.</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="n">
+        <v>4</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2135,17 +2391,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Higher cost for maintenance and logistical support required.</t>
+          <t>Higher costs for maintenance and logistical support due to complex supply chain and remote operations.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Assembly and commissioning</t>
+          <t>Normal Power Production</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2159,7 +2415,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H34" t="n">
         <v>4</v>
@@ -2171,12 +2427,20 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Developing system requirements with local and 3rd party input, training leads, and structuring contracts with incentives/penalties and FFP.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
+          <t>Structure contracts to include incentives/penalties and firm-fixed-price elements where possible.</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>